<commit_message>
Add data checks, backtest, what-if simulator, daily brief and rebuttal builder
New pages: Data Check, Backtest, What-If Simulator, Rebuttal Builder, Daily Brief.
Telugu replies for Ask AI, speeches and rebuttals.

Data Check cross-validates the sheets (shares add up, deltas match the share
tables, official votes match percentages) and flags a point written under one
party's column that names another party's candidate. It found Gopinath's point
filed under Congress; Book 13.xlsx now has it under BRS (two cell references
changed, nothing else in the workbook touched).

Ask AI and Rebuttal prompts now refuse to tie a fact to a voter group unless
the data does, and treat promises as promises. AUTH_DISABLED secret lets the
password lock be switched off explicitly for testing; it stays on by default.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Book 13.xlsx
+++ b/Book 13.xlsx
@@ -6248,10 +6248,10 @@
         <v>128</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" t="s">
         <v>129</v>
-      </c>
-      <c r="D7" t="s">
-        <v>130</v>
       </c>
       <c r="E7" t="s">
         <v>130</v>

</xml_diff>

<commit_message>
Add Mood Check, freshness labels, 2025 by-election result and accuracy fixes
Result-aware pages, mood guard, sample-weighted survey blend, NaN-safe conflict check, model switch to gpt-4.1-mini.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Book 13.xlsx
+++ b/Book 13.xlsx
@@ -4196,8 +4196,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{116844CD-DE7C-43A5-9170-A2DCB5030632}" name="Table6" displayName="Table6" ref="A1:F6" totalsRowShown="0" headerRowDxfId="10">
-  <autoFilter ref="A1:F6" xr:uid="{116844CD-DE7C-43A5-9170-A2DCB5030632}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{116844CD-DE7C-43A5-9170-A2DCB5030632}" name="Table6" displayName="Table6" ref="A1:F9" totalsRowShown="0" headerRowDxfId="10">
+  <autoFilter ref="A1:F9" xr:uid="{116844CD-DE7C-43A5-9170-A2DCB5030632}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{E4793850-1094-4D47-BE85-026FF6FDF225}" name="Year"/>
     <tableColumn id="2" xr3:uid="{5BC23BD4-36F8-4518-8EBC-B17002E9BF7E}" name="Party"/>
@@ -5648,7 +5648,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB4A6BF-BAFA-4ADC-8670-F72774953FB8}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
@@ -5773,6 +5773,72 @@
       </c>
       <c r="F6" s="5">
         <v>165368</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>2025</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Vallala Naveen Yadav</t>
+        </is>
+      </c>
+      <c r="D7" s="5">
+        <v>98988</v>
+      </c>
+      <c r="E7">
+        <v>50.83</v>
+      </c>
+      <c r="F7" s="5">
+        <v>194727</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>2025</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Maganti Sunitha</t>
+        </is>
+      </c>
+      <c r="D8" s="5">
+        <v>74259</v>
+      </c>
+      <c r="E8">
+        <v>38.13</v>
+      </c>
+      <c r="F8" s="5">
+        <v>194727</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>2025</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lankala Deepak Reddy</t>
+        </is>
+      </c>
+      <c r="D9" s="5">
+        <v>17061</v>
+      </c>
+      <c r="E9">
+        <v>8.76</v>
+      </c>
+      <c r="F9" s="5">
+        <v>194727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>